<commit_message>
Version 2.5.9.0 se agregó mes al final del reporte de ventas, y se agregó un filtro de busqueda por número de factura.
</commit_message>
<xml_diff>
--- a/Jeic/Jeic/Resources/Plantilla.xlsx
+++ b/Jeic/Jeic/Resources/Plantilla.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boxbu\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/de8a898b81206ef9/Documents/JEIC PROYECTO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CA0671-9155-46F3-8043-A1558621FC92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{09CA0671-9155-46F3-8043-A1558621FC92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D78F94D6-31AE-4891-B980-63C504D43647}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>Fecha:</t>
   </si>
@@ -204,6 +204,9 @@
   </si>
   <si>
     <t>REALIZÓ BAJA</t>
+  </si>
+  <si>
+    <t>FECHA DE ASIGNACIÓN (MES)</t>
   </si>
 </sst>
 </file>
@@ -211,8 +214,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -300,17 +303,17 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -334,10 +337,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -351,9 +354,9 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Moneda" xfId="2" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -679,8 +682,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:BB9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:BC9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.6640625" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.109375" style="5" bestFit="1" customWidth="1"/>
@@ -736,15 +739,16 @@
     <col min="52" max="52" width="15" style="5" bestFit="1" customWidth="1"/>
     <col min="53" max="53" width="10.6640625" style="5" bestFit="1" customWidth="1"/>
     <col min="54" max="54" width="16.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="55" max="16384" width="8.88671875" style="5"/>
+    <col min="55" max="55" width="26.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="56" max="16384" width="8.88671875" style="5"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:54" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:55" x14ac:dyDescent="0.3">
       <c r="L2" s="6" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:54" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:55" x14ac:dyDescent="0.3">
       <c r="F3" s="15" t="s">
         <v>35</v>
       </c>
@@ -754,7 +758,7 @@
       <c r="J3" s="15"/>
       <c r="K3" s="15"/>
     </row>
-    <row r="8" spans="1:54" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:55" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -917,8 +921,11 @@
       <c r="BB8" s="7" t="s">
         <v>54</v>
       </c>
+      <c r="BC8" s="7" t="s">
+        <v>57</v>
+      </c>
     </row>
-    <row r="9" spans="1:54" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:55" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>34</v>
       </c>

</xml_diff>

<commit_message>
Version 2.6.0.0 se agregan los dias de credito en el formulario de factura y en el reporte de ventas.
</commit_message>
<xml_diff>
--- a/Jeic/Jeic/Resources/Plantilla.xlsx
+++ b/Jeic/Jeic/Resources/Plantilla.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/de8a898b81206ef9/Documents/JEIC PROYECTO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{09CA0671-9155-46F3-8043-A1558621FC92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D78F94D6-31AE-4891-B980-63C504D43647}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{09CA0671-9155-46F3-8043-A1558621FC92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{040B698C-4F66-45FE-A0B3-FC529C1BAD70}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plantilla" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>Fecha:</t>
   </si>
@@ -207,6 +207,9 @@
   </si>
   <si>
     <t>FECHA DE ASIGNACIÓN (MES)</t>
+  </si>
+  <si>
+    <t>ESTADO FACTURA</t>
   </si>
 </sst>
 </file>
@@ -417,6 +420,10 @@
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -682,7 +689,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:BC9"/>
+  <dimension ref="A2:BD9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.6640625" style="5" bestFit="1" customWidth="1"/>
@@ -739,16 +746,16 @@
     <col min="52" max="52" width="15" style="5" bestFit="1" customWidth="1"/>
     <col min="53" max="53" width="10.6640625" style="5" bestFit="1" customWidth="1"/>
     <col min="54" max="54" width="16.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="26.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="56" max="16384" width="8.88671875" style="5"/>
+    <col min="55" max="56" width="26.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="57" max="16384" width="8.88671875" style="5"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:55" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:56" x14ac:dyDescent="0.3">
       <c r="L2" s="6" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:55" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:56" x14ac:dyDescent="0.3">
       <c r="F3" s="15" t="s">
         <v>35</v>
       </c>
@@ -758,7 +765,7 @@
       <c r="J3" s="15"/>
       <c r="K3" s="15"/>
     </row>
-    <row r="8" spans="1:55" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:56" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -924,8 +931,11 @@
       <c r="BC8" s="7" t="s">
         <v>57</v>
       </c>
+      <c r="BD8" s="7" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="9" spans="1:55" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:56" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>34</v>
       </c>

</xml_diff>